<commit_message>
Traitement RUP automatique : Boom (2850)
</commit_message>
<xml_diff>
--- a/state/2850_boom_rup.xlsx
+++ b/state/2850_boom_rup.xlsx
@@ -519,7 +519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T49"/>
+  <dimension ref="A1:U56"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
     <col width="18.42578125" customWidth="1" min="1" max="1"/>
@@ -656,6 +656,11 @@
           <t>Zone voor KMO</t>
         </is>
       </c>
+      <c r="U2" s="18" t="inlineStr">
+        <is>
+          <t>Zone voor Nieuwe Potaardestraat</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="42" customHeight="1">
       <c r="A3" s="11" t="n"/>
@@ -743,6 +748,13 @@
           <t>/</t>
         </is>
       </c>
+      <c r="U3" s="19" t="inlineStr">
+        <is>
+          <t>Bestemming
+Waar een zone voor nieuwe Potaardestraat is aangegeven kan wegeninfrastructuur
+aangelegd, beheerd en geëxploiteerd.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="20" t="inlineStr">
@@ -845,6 +857,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="B5" t="inlineStr">
@@ -942,6 +959,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="B6" t="inlineStr">
@@ -1039,6 +1061,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="B7" t="inlineStr">
@@ -1136,6 +1163,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="B8" t="inlineStr">
@@ -1233,6 +1265,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="B9" t="inlineStr">
@@ -1330,6 +1367,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="B10" t="inlineStr">
@@ -1427,6 +1469,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="B11" t="inlineStr">
@@ -1524,6 +1571,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="B12" t="inlineStr">
@@ -1621,6 +1673,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="B13" t="inlineStr">
@@ -1718,6 +1775,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="B14" t="inlineStr">
@@ -1815,6 +1877,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="B15" t="inlineStr">
@@ -1912,6 +1979,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="B16" t="inlineStr">
@@ -2009,6 +2081,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="B17" t="inlineStr">
@@ -2106,6 +2183,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="B18" t="inlineStr">
@@ -2203,6 +2285,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="B19" t="inlineStr">
@@ -2300,6 +2387,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="B20" t="inlineStr">
@@ -2397,6 +2489,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="B21" t="inlineStr">
@@ -2494,6 +2591,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="B22" t="inlineStr">
@@ -2591,6 +2693,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="B23" t="inlineStr">
@@ -2688,6 +2795,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="B24" t="inlineStr">
@@ -2785,6 +2897,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="B25" t="inlineStr">
@@ -2882,6 +2999,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="B26" t="inlineStr">
@@ -2979,6 +3101,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="B27" t="inlineStr">
@@ -3076,6 +3203,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="B28" t="inlineStr">
@@ -3173,6 +3305,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="B29" t="inlineStr">
@@ -3270,6 +3407,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="B30" t="inlineStr">
@@ -3367,6 +3509,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="B31" t="inlineStr">
@@ -3464,6 +3611,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="20" t="inlineStr">
@@ -3566,6 +3718,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="B33" t="inlineStr">
@@ -3663,6 +3820,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="B34" t="inlineStr">
@@ -3760,6 +3922,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="B35" t="inlineStr">
@@ -3857,6 +4024,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="B36" t="inlineStr">
@@ -3954,6 +4126,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="20" t="inlineStr">
@@ -4056,6 +4233,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="B38" t="inlineStr">
@@ -4153,6 +4335,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="20" t="inlineStr">
@@ -4255,6 +4442,11 @@
           <t>O</t>
         </is>
       </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="B40" t="inlineStr">
@@ -4352,6 +4544,11 @@
           <t>O</t>
         </is>
       </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="B41" t="inlineStr">
@@ -4449,6 +4646,11 @@
           <t>O</t>
         </is>
       </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="B42" t="inlineStr">
@@ -4546,6 +4748,11 @@
           <t>O</t>
         </is>
       </c>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="B43" t="inlineStr">
@@ -4643,6 +4850,11 @@
           <t>O</t>
         </is>
       </c>
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="B44" t="inlineStr">
@@ -4740,6 +4952,11 @@
           <t>O</t>
         </is>
       </c>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="B45" t="inlineStr">
@@ -4837,6 +5054,11 @@
           <t>O</t>
         </is>
       </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="B46" t="inlineStr">
@@ -4934,6 +5156,11 @@
           <t>O</t>
         </is>
       </c>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="B47" t="inlineStr">
@@ -5031,6 +5258,11 @@
           <t>O</t>
         </is>
       </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="B48" t="inlineStr">
@@ -5128,14 +5360,733 @@
           <t>N</t>
         </is>
       </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
-    <row r="49"/>
+    <row r="49">
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Boom</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>2850</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Klampovenweg</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>241H</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>https://dsi.omgeving.vlaanderen.be/fiche-detail/4c21479f-775a-476f-86d7-7b68365822e9</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>RUP_10000_213_00031_00001</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Boom</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>2850</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Klampovenweg</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>253F</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>https://dsi.omgeving.vlaanderen.be/fiche-detail/4c21479f-775a-476f-86d7-7b68365822e9</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>RUP_10000_213_00031_00001</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Boom</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>2850</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Klampovenweg</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>251D</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>https://dsi.omgeving.vlaanderen.be/fiche-detail/4c21479f-775a-476f-86d7-7b68365822e9</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>RUP_10000_213_00031_00001</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="U51" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Boom</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>2850</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Klampovenweg</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>243A</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>https://dsi.omgeving.vlaanderen.be/fiche-detail/4c21479f-775a-476f-86d7-7b68365822e9</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>RUP_10000_213_00031_00001</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="U52" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Boom</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>2850</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Klampovenweg</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>251C</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>https://dsi.omgeving.vlaanderen.be/fiche-detail/4c21479f-775a-476f-86d7-7b68365822e9</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>RUP_10000_213_00031_00001</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="U53" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Boom</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>2850</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Klampovenweg</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>303A</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>https://dsi.omgeving.vlaanderen.be/fiche-detail/4c21479f-775a-476f-86d7-7b68365822e9</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>RUP_10000_213_00031_00001</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="T54" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="U54" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Boom</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>2850</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Klampovenweg</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>303K</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>https://dsi.omgeving.vlaanderen.be/fiche-detail/4c21479f-775a-476f-86d7-7b68365822e9</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>RUP_10000_213_00031_00001</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="T55" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="U55" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="56"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A37:A38"/>
     <mergeCell ref="A32:A36"/>
-    <mergeCell ref="A39:A48"/>
     <mergeCell ref="A4:A31"/>
+    <mergeCell ref="A39:A55"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>